<commit_message>
feat: Enhance workdesk meta and task management features
- Updated `getWorkdeskMeta` to include comprehensive workflow statuses based on user roles.
- Expanded `workdeskTask.controller.js` to support new task attributes including work levels, job work statuses, and additional financial fields.
- Implemented task job work status updates and validation for task status transitions.
- Introduced new utility functions for lead and mail synchronization, ensuring data consistency across models.
- Enhanced client model to support additional portal credentials and improved client ID generation logic.
- Updated validation schemas to accommodate new fields in client and task models.
- Added bulk synchronization for leads and mails to streamline data management.
- Introduced new fields in the invoice model for better financial tracking.
- Updated routes to simplify client and task management operations.
</commit_message>
<xml_diff>
--- a/src/static/sample-leads.xlsx
+++ b/src/static/sample-leads.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="SampleLeads" sheetId="1" r:id="rId1"/>
+    <sheet name="Sample" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AM1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -473,15 +473,54 @@
         <v>leadStatus</v>
       </c>
       <c r="Y1" t="str">
+        <v>senderEmail</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>emailVerifiedStatus</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>wifi</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>browser</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>emailSentOn</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>emailTemplate</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>emailSubjectCode</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>emailSeen</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>emailStatus</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>enquiryStatus</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>turnup</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>cdcrNo</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>cdcrCreation</v>
+      </c>
+      <c r="AL1" t="str">
         <v>description</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AM1" t="str">
         <v>notes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>